<commit_message>
docs(docs): record that the dogfood run executed main's code, so 049's live gate moves past the merge
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/features/049-preview-environment-gate/testing-plan.xlsx
+++ b/docs/features/049-preview-environment-gate/testing-plan.xlsx
@@ -1466,11 +1466,19 @@
           <t>'preview environment: not required — no apps/*frontend* or apps/*backend* directory'</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Not observable on this PR: dogfood.yml passes no ql-pipeline-ref, so the govern step checks ql-pipeline out at main and ran 0.5.1's code against this branch. The log carries 'task artifacts: complete' and no preview line.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Gate 3 - read the checks / ql-pipeline log after the push</t>
+          <t>Gate 3 moves to the first governed run after #43 merges. Filed separately: dogfood should pass ql-pipeline-ref: github.head_ref so a PR exercises its own code.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>

</xml_diff>